<commit_message>
Migrate design from wknd-trendsetters.site and fix FAQ hero import
Phase 1 (site design) verified and Phase 2 block styling migrated to match
the source across all 10 site blocks (95-98% visual match): accordion-faq,
banner-cta, cards-article, cards-gallery, cards-trend, columns-article,
columns-contact, columns-feature, columns-intro, tabs-testimonial.

Notable changes:
- banner-cta rebuilt as a rounded photo card with gradient overlay (image
  was previously dropped)
- accordion-faq open-state icon now rotates + into x
- corrected card image aspect ratios and responsive breakpoints

Post-critique fix:
- columns-intro parser now captures all paragraphs in the hero content column
  (was querySelector, dropping the FAQ hero lead paragraph); rebuilt the FAQ
  import bundle and re-imported so faq.plain.html includes the missing line

Also fixed pre-existing lint errors in article-list and employee-list blocks.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-faq-page.report.xlsx
+++ b/tools/importer/reports/import-faq-page.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="100">
   <si>
     <t>_reportFile</t>
   </si>
@@ -109,7 +109,7 @@
     <t>faq-page</t>
   </si>
   <si>
-    <t>2026-09-02T12:08:10.562Z</t>
+    <t>2026-09-02T20:06:02.435Z</t>
   </si>
   <si>
     <t>FAQ - The Fashion Blog</t>
@@ -149,6 +149,27 @@
   </si>
   <si>
     <t>https://wknd-trendsetters.site/fashion-trends-of-the-season</t>
+  </si>
+  <si>
+    <t>fashion-trends-young-adults-casual-sport.report.json</t>
+  </si>
+  <si>
+    <t>["columns-intro","cards-trend","columns-feature"]</t>
+  </si>
+  <si>
+    <t>fashion-trends-young-adults-casual-sport</t>
+  </si>
+  <si>
+    <t>trends-showcase</t>
+  </si>
+  <si>
+    <t>2026-09-02T12:34:38.511Z</t>
+  </si>
+  <si>
+    <t>Fashion Trends for Young Adults | Fashion Blog</t>
+  </si>
+  <si>
+    <t>https://wknd-trendsetters.site/fashion-trends-young-adults-casual-sport</t>
   </si>
   <si>
     <t>fashion-trends-young-adults.report.json</t>
@@ -678,11 +699,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="41" customWidth="1"/>
+    <col min="3" max="3" width="42" customWidth="1"/>
     <col min="5" max="5" width="17" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="8" width="50" customWidth="1"/>
@@ -884,27 +905,27 @@
         <v>11</v>
       </c>
       <c r="E8" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="F8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B9" t="s">
-        <v>9</v>
+        <v>54</v>
       </c>
       <c r="C9" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
@@ -913,36 +934,36 @@
         <v>42</v>
       </c>
       <c r="F9" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="G9" t="s">
-        <v>13</v>
+        <v>57</v>
       </c>
       <c r="H9" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B10" t="s">
-        <v>57</v>
+        <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D10" t="s">
         <v>11</v>
       </c>
       <c r="E10" t="s">
-        <v>59</v>
+        <v>42</v>
       </c>
       <c r="F10" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G10" t="s">
-        <v>61</v>
+        <v>13</v>
       </c>
       <c r="H10" t="s">
         <v>62</v>
@@ -953,155 +974,181 @@
         <v>63</v>
       </c>
       <c r="B11" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="C11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D11" t="s">
         <v>11</v>
       </c>
       <c r="E11" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="F11" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="G11" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B12" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="C12" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D12" t="s">
         <v>11</v>
       </c>
       <c r="E12" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="F12" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G12" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B13" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="C13" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D13" t="s">
         <v>11</v>
       </c>
       <c r="E13" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="F13" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G13" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B14" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="C14" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D14" t="s">
         <v>11</v>
       </c>
       <c r="E14" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="F14" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G14" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="H14" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B15" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="C15" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D15" t="s">
         <v>11</v>
       </c>
       <c r="E15" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="F15" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="G15" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="H15" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B16" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="C16" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D16" t="s">
         <v>11</v>
       </c>
       <c r="E16" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="F16" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G16" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="H16" t="s">
-        <v>92</v>
+        <v>94</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>95</v>
+      </c>
+      <c r="B17" t="s">
+        <v>64</v>
+      </c>
+      <c r="C17" t="s">
+        <v>96</v>
+      </c>
+      <c r="D17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17" t="s">
+        <v>66</v>
+      </c>
+      <c r="F17" t="s">
+        <v>97</v>
+      </c>
+      <c r="G17" t="s">
+        <v>98</v>
+      </c>
+      <c r="H17" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>